<commit_message>
Preserve original values in rollup workbook
Co-authored-by: ScheelJW <ScheelJW@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/5 MXG 2 Year Accident_Abuse.xlsx
+++ b/5 MXG 2 Year Accident_Abuse.xlsx
@@ -79,9 +79,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -91,16 +91,10 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -520,11 +514,11 @@
   <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -534,11 +528,11 @@
           <t>5 MXG 2 Year Accident/Abuse Summary Rollup</t>
         </is>
       </c>
-      <c r="B1" s="1" t="n"/>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n"/>
@@ -611,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>36471.38</v>
+        <v>36306.38</v>
       </c>
       <c r="C7" s="2" t="n"/>
       <c r="D7" s="2" t="n"/>
@@ -667,460 +661,460 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>23 BGS</t>
         </is>
       </c>
-      <c r="B11" s="6" t="n">
+      <c r="B11" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="C11" s="6" t="n">
+      <c r="C11" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="D11" s="6" t="n">
+      <c r="D11" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="E11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="7" t="n">
+      <c r="E11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="3" t="n">
         <v>2158.49</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>23 BGS</t>
         </is>
       </c>
-      <c r="B12" s="6" t="n">
+      <c r="B12" s="2" t="n">
         <v>2025</v>
       </c>
-      <c r="C12" s="6" t="n">
+      <c r="C12" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="D12" s="6" t="n">
+      <c r="D12" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="E12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="7" t="n">
+      <c r="E12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="3" t="n">
         <v>4720.52</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>5 AMXS</t>
         </is>
       </c>
-      <c r="B13" s="6" t="n">
+      <c r="B13" s="2" t="n">
         <v>2023</v>
       </c>
-      <c r="C13" s="6" t="n">
+      <c r="C13" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D13" s="6" t="n">
+      <c r="D13" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="E13" s="6" t="n">
+      <c r="E13" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="F13" s="7" t="n">
-        <v>5465.82</v>
+      <c r="F13" s="3" t="n">
+        <v>5300.82</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>5 AMXS</t>
         </is>
       </c>
-      <c r="B14" s="6" t="n">
+      <c r="B14" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="C14" s="6" t="n">
+      <c r="C14" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="D14" s="6" t="n">
+      <c r="D14" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="E14" s="6" t="n">
+      <c r="E14" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="F14" s="7" t="n">
+      <c r="F14" s="3" t="n">
         <v>5719.570000000001</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>5 AMXS</t>
         </is>
       </c>
-      <c r="B15" s="6" t="n">
+      <c r="B15" s="2" t="n">
         <v>2025</v>
       </c>
-      <c r="C15" s="6" t="n">
+      <c r="C15" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D15" s="6" t="n">
+      <c r="D15" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E15" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" s="7" t="n">
+      <c r="E15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>5 MUNS</t>
         </is>
       </c>
-      <c r="B16" s="6" t="n">
+      <c r="B16" s="2" t="n">
         <v>2023</v>
       </c>
-      <c r="C16" s="6" t="n">
+      <c r="C16" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D16" s="6" t="n">
+      <c r="D16" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E16" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="7" t="n">
+      <c r="E16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>5 MUNS</t>
         </is>
       </c>
-      <c r="B17" s="6" t="n">
+      <c r="B17" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="C17" s="6" t="n">
+      <c r="C17" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="D17" s="6" t="n">
+      <c r="D17" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="E17" s="6" t="n">
+      <c r="E17" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="F17" s="7" t="n">
+      <c r="F17" s="3" t="n">
         <v>2328</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>5 MUNS</t>
         </is>
       </c>
-      <c r="B18" s="6" t="n">
+      <c r="B18" s="2" t="n">
         <v>2025</v>
       </c>
-      <c r="C18" s="6" t="n">
+      <c r="C18" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="D18" s="6" t="n">
+      <c r="D18" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E18" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" s="7" t="n">
+      <c r="E18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="3" t="n">
         <v>91.70999999999999</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>5 MUNS</t>
         </is>
       </c>
-      <c r="B19" s="6" t="n">
+      <c r="B19" s="2" t="n">
         <v>2026</v>
       </c>
-      <c r="C19" s="6" t="n">
+      <c r="C19" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D19" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="7" t="n">
+      <c r="D19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>5 MXG</t>
         </is>
       </c>
-      <c r="B20" s="6" t="n">
+      <c r="B20" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="C20" s="6" t="n">
+      <c r="C20" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D20" s="6" t="n">
+      <c r="D20" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E20" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" s="7" t="n">
+      <c r="E20" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>5 MXG</t>
         </is>
       </c>
-      <c r="B21" s="6" t="n">
+      <c r="B21" s="2" t="n">
         <v>2025</v>
       </c>
-      <c r="C21" s="6" t="n">
+      <c r="C21" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D21" s="6" t="n">
+      <c r="D21" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E21" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" s="7" t="n">
+      <c r="E21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>5 MXS</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="n">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>5 MXS</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
         <v>2023</v>
       </c>
-      <c r="C22" s="6" t="n">
+      <c r="C22" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D22" s="6" t="n">
+      <c r="D22" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E22" s="6" t="n">
+      <c r="E22" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="F22" s="7" t="n">
+      <c r="F22" s="3" t="n">
         <v>1045.8</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>5 MXS</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="n">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>5 MXS</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="C23" s="6" t="n">
+      <c r="C23" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="D23" s="6" t="n">
+      <c r="D23" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="E23" s="6" t="n">
+      <c r="E23" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="F23" s="7" t="n">
+      <c r="F23" s="3" t="n">
         <v>12555</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>5 MXS</t>
-        </is>
-      </c>
-      <c r="B24" s="6" t="n">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>5 MXS</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n">
         <v>2025</v>
       </c>
-      <c r="C24" s="6" t="n">
+      <c r="C24" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="D24" s="6" t="n">
+      <c r="D24" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="E24" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" s="7" t="n">
+      <c r="E24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="3" t="n">
         <v>2086.47</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>5 MXS</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="n">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>5 MXS</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n">
         <v>2026</v>
       </c>
-      <c r="C25" s="6" t="n">
+      <c r="C25" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D25" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" s="7" t="n">
+      <c r="D25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>5 OSS</t>
         </is>
       </c>
-      <c r="B26" s="6" t="n">
+      <c r="B26" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="C26" s="6" t="n">
+      <c r="C26" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D26" s="6" t="n">
+      <c r="D26" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E26" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F26" s="7" t="n">
+      <c r="E26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="inlineStr">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>69 BGS</t>
         </is>
       </c>
-      <c r="B27" s="6" t="n">
+      <c r="B27" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="C27" s="6" t="n">
+      <c r="C27" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D27" s="6" t="n">
+      <c r="D27" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="E27" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F27" s="7" t="n">
+      <c r="E27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="inlineStr">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>69 BGS</t>
         </is>
       </c>
-      <c r="B28" s="6" t="n">
+      <c r="B28" s="2" t="n">
         <v>2026</v>
       </c>
-      <c r="C28" s="6" t="n">
+      <c r="C28" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D28" s="6" t="n">
+      <c r="D28" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E28" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F28" s="7" t="n">
+      <c r="E28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="6" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>705 MUNS</t>
         </is>
       </c>
-      <c r="B29" s="6" t="n">
+      <c r="B29" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="C29" s="6" t="n">
+      <c r="C29" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="D29" s="6" t="n">
+      <c r="D29" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="E29" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F29" s="7" t="n">
+      <c r="E29" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="3" t="n">
         <v>300</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="inlineStr">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>705 MUNS</t>
         </is>
       </c>
-      <c r="B30" s="6" t="n">
+      <c r="B30" s="2" t="n">
         <v>2025</v>
       </c>
-      <c r="C30" s="6" t="n">
+      <c r="C30" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="D30" s="6" t="n">
+      <c r="D30" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E30" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F30" s="7" t="n">
+      <c r="E30" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="n"/>
-      <c r="B31" s="6" t="n"/>
-      <c r="C31" s="6" t="n"/>
-      <c r="D31" s="6" t="n"/>
-      <c r="E31" s="6" t="n"/>
-      <c r="F31" s="7" t="n"/>
+      <c r="A31" s="2" t="n"/>
+      <c r="B31" s="2" t="n"/>
+      <c r="C31" s="2" t="n"/>
+      <c r="D31" s="2" t="n"/>
+      <c r="E31" s="2" t="n"/>
+      <c r="F31" s="3" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="n"/>
-      <c r="B32" s="6" t="n"/>
-      <c r="C32" s="6" t="n"/>
-      <c r="D32" s="6" t="n"/>
-      <c r="E32" s="6" t="n"/>
-      <c r="F32" s="7" t="n"/>
+      <c r="A32" s="2" t="n"/>
+      <c r="B32" s="2" t="n"/>
+      <c r="C32" s="2" t="n"/>
+      <c r="D32" s="2" t="n"/>
+      <c r="E32" s="2" t="n"/>
+      <c r="F32" s="3" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -1148,171 +1142,171 @@
           <t>Total Cost</t>
         </is>
       </c>
-      <c r="F33" s="7" t="n"/>
+      <c r="F33" s="3" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="6" t="inlineStr">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>23 BGS</t>
         </is>
       </c>
-      <c r="B34" s="6" t="n">
+      <c r="B34" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="C34" s="6" t="n">
+      <c r="C34" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="D34" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E34" s="7" t="n">
+      <c r="D34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" s="3" t="n">
         <v>6879.01</v>
       </c>
-      <c r="F34" s="7" t="n"/>
+      <c r="F34" s="3" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="6" t="inlineStr">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>5 AMXS</t>
         </is>
       </c>
-      <c r="B35" s="6" t="n">
+      <c r="B35" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="C35" s="6" t="n">
+      <c r="C35" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="D35" s="6" t="n">
+      <c r="D35" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="E35" s="7" t="n">
-        <v>11185.39</v>
-      </c>
-      <c r="F35" s="7" t="n"/>
+      <c r="E35" s="3" t="n">
+        <v>11020.39</v>
+      </c>
+      <c r="F35" s="3" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="6" t="inlineStr">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>5 MUNS</t>
         </is>
       </c>
-      <c r="B36" s="6" t="n">
+      <c r="B36" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="C36" s="6" t="n">
+      <c r="C36" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="D36" s="6" t="n">
+      <c r="D36" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E36" s="7" t="n">
+      <c r="E36" s="3" t="n">
         <v>2419.71</v>
       </c>
-      <c r="F36" s="7" t="n"/>
+      <c r="F36" s="3" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="6" t="inlineStr">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>5 MXG</t>
         </is>
       </c>
-      <c r="B37" s="6" t="n">
+      <c r="B37" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C37" s="6" t="n">
+      <c r="C37" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D37" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E37" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F37" s="7" t="n"/>
+      <c r="D37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" s="3" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="6" t="inlineStr">
-        <is>
-          <t>5 MXS</t>
-        </is>
-      </c>
-      <c r="B38" s="6" t="n">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>5 MXS</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="n">
         <v>37</v>
       </c>
-      <c r="C38" s="6" t="n">
+      <c r="C38" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="D38" s="6" t="n">
+      <c r="D38" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="E38" s="7" t="n">
+      <c r="E38" s="3" t="n">
         <v>15687.27</v>
       </c>
-      <c r="F38" s="7" t="n"/>
+      <c r="F38" s="3" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="6" t="inlineStr">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>5 OSS</t>
         </is>
       </c>
-      <c r="B39" s="6" t="n">
+      <c r="B39" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C39" s="6" t="n">
+      <c r="C39" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D39" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E39" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F39" s="7" t="n"/>
+      <c r="D39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" s="3" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="6" t="inlineStr">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>69 BGS</t>
         </is>
       </c>
-      <c r="B40" s="6" t="n">
+      <c r="B40" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="C40" s="6" t="n">
+      <c r="C40" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="D40" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E40" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F40" s="7" t="n"/>
+      <c r="D40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="3" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="6" t="inlineStr">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>705 MUNS</t>
         </is>
       </c>
-      <c r="B41" s="6" t="n">
+      <c r="B41" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="C41" s="6" t="n">
+      <c r="C41" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="D41" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E41" s="7" t="n">
+      <c r="D41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" s="3" t="n">
         <v>300</v>
       </c>
-      <c r="F41" s="7" t="n"/>
+      <c r="F41" s="3" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="2">
@@ -1343,47 +1337,47 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Reg#</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Veh type</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Assigned Org</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Billed Org</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Case number</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>Description of damage</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>Date Opened</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>Cost</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>Date Closed</t>
         </is>
@@ -1395,9 +1389,10 @@
           <t>10B02060</t>
         </is>
       </c>
-      <c r="B2" s="2">
-        <f>VLOOKUP(A2,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>CHE MLT</t>
+        </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -1419,13 +1414,13 @@
           <t>WIND DAMAGE TO BOTH FRONT DOORS AND UNREPORTED DAMAGE TO SLIDING DOOR WINDOW GLASS</t>
         </is>
       </c>
-      <c r="G2" s="8" t="n">
+      <c r="G2" s="6" t="n">
         <v>45223</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>3022.35</v>
       </c>
-      <c r="I2" s="8" t="n">
+      <c r="I2" s="6" t="n">
         <v>45286</v>
       </c>
     </row>
@@ -1435,9 +1430,10 @@
           <t>08B01137</t>
         </is>
       </c>
-      <c r="B3" s="2">
-        <f>VLOOKUP(A3,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>CHE P/U</t>
+        </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -1459,13 +1455,13 @@
           <t>wind damage and unreported damage to RF DOOR, AND inside door handle, dent in lr cargo box in front of wheel</t>
         </is>
       </c>
-      <c r="G3" s="8" t="n">
+      <c r="G3" s="6" t="n">
         <v>45244</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>306.84</v>
-      </c>
-      <c r="I3" s="8" t="n">
+        <v>141.84</v>
+      </c>
+      <c r="I3" s="6" t="n">
         <v>45267</v>
       </c>
     </row>
@@ -1475,9 +1471,10 @@
           <t>16B00104</t>
         </is>
       </c>
-      <c r="B4" s="2">
-        <f>VLOOKUP(A4,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>FRD/VAN</t>
+        </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
@@ -1499,13 +1496,13 @@
           <t>see sf-91 for explanation but it looks like wind damage to rf door and fender</t>
         </is>
       </c>
-      <c r="G4" s="8" t="n">
+      <c r="G4" s="6" t="n">
         <v>45246</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>545.13</v>
       </c>
-      <c r="I4" s="8" t="n">
+      <c r="I4" s="6" t="n">
         <v>45286</v>
       </c>
     </row>
@@ -1515,9 +1512,10 @@
           <t>16C00117</t>
         </is>
       </c>
-      <c r="B5" s="2">
-        <f>VLOOKUP(A5,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>FRD B/T</t>
+        </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
@@ -1539,13 +1537,13 @@
           <t>BLOCK HEATER CORD TORN OFF</t>
         </is>
       </c>
-      <c r="G5" s="8" t="n">
+      <c r="G5" s="6" t="n">
         <v>45260</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I5" s="8" t="n"/>
+      <c r="I5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1553,9 +1551,10 @@
           <t>07C00267</t>
         </is>
       </c>
-      <c r="B6" s="2">
-        <f>VLOOKUP(A6,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>FRD BOBTAIL</t>
+        </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -1577,13 +1576,13 @@
           <t>ORG TIED CHAIN AROUND DRAGLINK/TIE ROD INSTEAD OF TOW HOOK, BENT DRAG LINK AND TOR ROD ARM</t>
         </is>
       </c>
-      <c r="G6" s="8" t="n">
+      <c r="G6" s="6" t="n">
         <v>45271</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>500.67</v>
       </c>
-      <c r="I6" s="8" t="n">
+      <c r="I6" s="6" t="n">
         <v>45303</v>
       </c>
     </row>
@@ -1593,9 +1592,10 @@
           <t>10B02067</t>
         </is>
       </c>
-      <c r="B7" s="2">
-        <f>VLOOKUP(A7,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>CHE MLT</t>
+        </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
@@ -1617,13 +1617,13 @@
           <t>wind damage to left front door</t>
         </is>
       </c>
-      <c r="G7" s="8" t="n">
+      <c r="G7" s="6" t="n">
         <v>45272</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>857.42</v>
       </c>
-      <c r="I7" s="8" t="n">
+      <c r="I7" s="6" t="n">
         <v>45303</v>
       </c>
     </row>
@@ -1633,9 +1633,10 @@
           <t>16C00103</t>
         </is>
       </c>
-      <c r="B8" s="2">
-        <f>VLOOKUP(A8,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>FRD B/T</t>
+        </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -1657,13 +1658,13 @@
           <t>notify only, waiver minor chip in left door mirror plastic housing</t>
         </is>
       </c>
-      <c r="G8" s="8" t="n">
+      <c r="G8" s="6" t="n">
         <v>45272</v>
       </c>
       <c r="H8" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I8" s="8" t="n"/>
+      <c r="I8" s="6" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1671,9 +1672,10 @@
           <t>11B01316</t>
         </is>
       </c>
-      <c r="B9" s="2">
-        <f>VLOOKUP(A9,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>CHE MLT</t>
+        </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -1695,13 +1697,13 @@
           <t>WIND DAMAGE TO RF DOOR AND FENDER</t>
         </is>
       </c>
-      <c r="G9" s="8" t="n">
+      <c r="G9" s="6" t="n">
         <v>45278</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>768.96</v>
       </c>
-      <c r="I9" s="8" t="n"/>
+      <c r="I9" s="6" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1709,9 +1711,10 @@
           <t>08B01139</t>
         </is>
       </c>
-      <c r="B10" s="2">
-        <f>VLOOKUP(A10,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>CHE P/U</t>
+        </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -1733,13 +1736,13 @@
           <t>unreported damage to left rear cargo box behind left tire//b/s pulled eent and touch up painted, no charge</t>
         </is>
       </c>
-      <c r="G10" s="8" t="n">
+      <c r="G10" s="6" t="n">
         <v>45313</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>135</v>
       </c>
-      <c r="I10" s="8" t="n"/>
+      <c r="I10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1747,9 +1750,10 @@
           <t>13C00072</t>
         </is>
       </c>
-      <c r="B11" s="2">
-        <f>VLOOKUP(A11,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>GLODET</t>
+        </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
@@ -1771,13 +1775,13 @@
           <t>boom red light broken</t>
         </is>
       </c>
-      <c r="G11" s="8" t="n">
+      <c r="G11" s="6" t="n">
         <v>45316</v>
       </c>
       <c r="H11" s="3" t="n">
         <v>310</v>
       </c>
-      <c r="I11" s="8" t="n">
+      <c r="I11" s="6" t="n">
         <v>45335</v>
       </c>
     </row>
@@ -1787,9 +1791,10 @@
           <t>10B02065</t>
         </is>
       </c>
-      <c r="B12" s="2">
-        <f>VLOOKUP(A12,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>CHE MLT</t>
+        </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
@@ -1811,14 +1816,14 @@
           <t>LEFT MIRROR HOUSING CRACKED</t>
         </is>
       </c>
-      <c r="G12" s="8" t="n">
+      <c r="G12" s="6" t="n">
         <v>45323</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>189.99</v>
       </c>
-      <c r="I12" s="8" t="n">
-        <v>45365</v>
+      <c r="I12" s="6" t="n">
+        <v>45370</v>
       </c>
     </row>
     <row r="13">
@@ -1827,9 +1832,10 @@
           <t>19L00597</t>
         </is>
       </c>
-      <c r="B13" s="2">
-        <f>VLOOKUP(A13,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>MB-2</t>
+        </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
@@ -1851,13 +1857,13 @@
           <t xml:space="preserve">left door mirror broken.  </t>
         </is>
       </c>
-      <c r="G13" s="8" t="n">
+      <c r="G13" s="6" t="n">
         <v>45323</v>
       </c>
       <c r="H13" s="3" t="n">
         <v>165.58</v>
       </c>
-      <c r="I13" s="8" t="n"/>
+      <c r="I13" s="6" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1865,9 +1871,10 @@
           <t>10B02069</t>
         </is>
       </c>
-      <c r="B14" s="2">
-        <f>VLOOKUP(A14,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>CHE MLT</t>
+        </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
@@ -1889,13 +1896,13 @@
           <t>turned in with 4 qts low on oil. Topped off oil level and sent notify letter to orgq</t>
         </is>
       </c>
-      <c r="G14" s="8" t="n">
+      <c r="G14" s="6" t="n">
         <v>45342</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I14" s="8" t="n"/>
+      <c r="I14" s="6" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1903,9 +1910,10 @@
           <t>12L01060</t>
         </is>
       </c>
-      <c r="B15" s="2">
-        <f>VLOOKUP(A15,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>NMC MB2</t>
+        </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
@@ -1927,13 +1935,13 @@
           <t>windshield cracked</t>
         </is>
       </c>
-      <c r="G15" s="8" t="n">
+      <c r="G15" s="6" t="n">
         <v>44999</v>
       </c>
       <c r="H15" s="3" t="n">
         <v>510.25</v>
       </c>
-      <c r="I15" s="8" t="n">
+      <c r="I15" s="6" t="n">
         <v>45390</v>
       </c>
     </row>
@@ -1943,9 +1951,10 @@
           <t>10B02067</t>
         </is>
       </c>
-      <c r="B16" s="2">
-        <f>VLOOKUP(A16,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>CHE MLT</t>
+        </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
@@ -1967,13 +1976,13 @@
           <t>heater box kicked in</t>
         </is>
       </c>
-      <c r="G16" s="8" t="n">
+      <c r="G16" s="6" t="n">
         <v>45373</v>
       </c>
       <c r="H16" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I16" s="8" t="n"/>
+      <c r="I16" s="6" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1981,9 +1990,10 @@
           <t>11B01316</t>
         </is>
       </c>
-      <c r="B17" s="2">
-        <f>VLOOKUP(A17,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>CHE MLT</t>
+        </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
@@ -2005,13 +2015,13 @@
           <t>WIND DAMAGE TO DOORS</t>
         </is>
       </c>
-      <c r="G17" s="8" t="n">
+      <c r="G17" s="6" t="n">
         <v>45390</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I17" s="8" t="n"/>
+      <c r="I17" s="6" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2019,9 +2029,10 @@
           <t>19L00597</t>
         </is>
       </c>
-      <c r="B18" s="2">
-        <f>VLOOKUP(A18,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>MB-2</t>
+        </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
@@ -2043,13 +2054,13 @@
           <t xml:space="preserve">OPERATOR OPENED DOOR AND PINS SNAPPED AND DOOR FELL OFF </t>
         </is>
       </c>
-      <c r="G18" s="8" t="n">
+      <c r="G18" s="6" t="n">
         <v>45432</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>414.2</v>
       </c>
-      <c r="I18" s="8" t="n">
+      <c r="I18" s="6" t="n">
         <v>45488</v>
       </c>
     </row>
@@ -2059,9 +2070,10 @@
           <t>08B01259</t>
         </is>
       </c>
-      <c r="B19" s="2">
-        <f>VLOOKUP(A19,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>CHE P/U</t>
+        </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
@@ -2083,13 +2095,13 @@
           <t>P/S FRONT AND REAR DOR DENTED, SCRATCHED PAINT</t>
         </is>
       </c>
-      <c r="G19" s="8" t="n">
+      <c r="G19" s="6" t="n">
         <v>45448</v>
       </c>
       <c r="H19" s="3" t="n">
         <v>4100.51</v>
       </c>
-      <c r="I19" s="8" t="n"/>
+      <c r="I19" s="6" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2097,9 +2109,10 @@
           <t>16L00044</t>
         </is>
       </c>
-      <c r="B20" s="2">
-        <f>VLOOKUP(A20,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>NMC MB-2</t>
+        </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
@@ -2121,13 +2134,13 @@
           <t>P/S MIRROR AND DOOR STRAP</t>
         </is>
       </c>
-      <c r="G20" s="8" t="n">
+      <c r="G20" s="6" t="n">
         <v>45450</v>
       </c>
       <c r="H20" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I20" s="8" t="n"/>
+      <c r="I20" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2135,9 +2148,10 @@
           <t>10B02061</t>
         </is>
       </c>
-      <c r="B21" s="2">
-        <f>VLOOKUP(A21,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>CHE MLT</t>
+        </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
@@ -2159,13 +2173,13 @@
           <t>WIND DAMAGE TO P/S DOOR</t>
         </is>
       </c>
-      <c r="G21" s="8" t="n">
+      <c r="G21" s="6" t="n">
         <v>45455</v>
       </c>
       <c r="H21" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I21" s="8" t="n"/>
+      <c r="I21" s="6" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2173,9 +2187,10 @@
           <t>11B01321</t>
         </is>
       </c>
-      <c r="B22" s="2">
-        <f>VLOOKUP(A22,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>CHE MLT</t>
+        </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
@@ -2197,13 +2212,13 @@
           <t xml:space="preserve">Heater Box </t>
         </is>
       </c>
-      <c r="G22" s="8" t="n">
+      <c r="G22" s="6" t="n">
         <v>45467</v>
       </c>
       <c r="H22" s="3" t="n">
         <v>404.29</v>
       </c>
-      <c r="I22" s="8" t="n"/>
+      <c r="I22" s="6" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2211,9 +2226,10 @@
           <t>10B02061</t>
         </is>
       </c>
-      <c r="B23" s="2">
-        <f>VLOOKUP(A23,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>CHE MLT</t>
+        </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
@@ -2235,13 +2251,13 @@
           <t xml:space="preserve">Wind damage </t>
         </is>
       </c>
-      <c r="G23" s="8" t="n">
+      <c r="G23" s="6" t="n">
         <v>45455</v>
       </c>
       <c r="H23" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I23" s="8" t="n"/>
+      <c r="I23" s="6" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2249,9 +2265,10 @@
           <t>11B01319</t>
         </is>
       </c>
-      <c r="B24" s="2">
-        <f>VLOOKUP(A24,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>CHE MLT</t>
+        </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
@@ -2273,13 +2290,13 @@
           <t>D/S REAR DOOR HINGE BENT/BROKE</t>
         </is>
       </c>
-      <c r="G24" s="8" t="n">
+      <c r="G24" s="6" t="n">
         <v>45544</v>
       </c>
       <c r="H24" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I24" s="8" t="n"/>
+      <c r="I24" s="6" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2287,9 +2304,10 @@
           <t>08B01884</t>
         </is>
       </c>
-      <c r="B25" s="2">
-        <f>VLOOKUP(A25,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>FTL TRC</t>
+        </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
@@ -2311,13 +2329,13 @@
           <t>exhaust stack bent</t>
         </is>
       </c>
-      <c r="G25" s="8" t="n">
+      <c r="G25" s="6" t="n">
         <v>45358</v>
       </c>
       <c r="H25" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I25" s="8" t="n"/>
+      <c r="I25" s="6" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2325,9 +2343,10 @@
           <t>08B01260</t>
         </is>
       </c>
-      <c r="B26" s="2">
-        <f>VLOOKUP(A26,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>CHE P/U</t>
+        </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
@@ -2349,13 +2368,13 @@
           <t>P/S FRONT DOOR DAMAGE</t>
         </is>
       </c>
-      <c r="G26" s="8" t="n">
+      <c r="G26" s="6" t="n">
         <v>45397</v>
       </c>
       <c r="H26" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I26" s="8" t="n"/>
+      <c r="I26" s="6" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2363,9 +2382,10 @@
           <t>10B00284</t>
         </is>
       </c>
-      <c r="B27" s="2">
-        <f>VLOOKUP(A27,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>FRD CGO</t>
+        </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
@@ -2387,13 +2407,13 @@
           <t>D/S BACK STEP BENT</t>
         </is>
       </c>
-      <c r="G27" s="8" t="n">
+      <c r="G27" s="6" t="n">
         <v>45531</v>
       </c>
       <c r="H27" s="3" t="n">
         <v>1164</v>
       </c>
-      <c r="I27" s="8" t="n">
+      <c r="I27" s="6" t="n">
         <v>45601</v>
       </c>
     </row>
@@ -2403,9 +2423,10 @@
           <t>08B01224</t>
         </is>
       </c>
-      <c r="B28" s="2">
-        <f>VLOOKUP(A28,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>CHE P/U</t>
+        </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
@@ -2427,13 +2448,13 @@
           <t>low on oil, topped off oil, no further engine damage, notify only</t>
         </is>
       </c>
-      <c r="G28" s="8" t="n">
+      <c r="G28" s="6" t="n">
         <v>45377</v>
       </c>
       <c r="H28" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I28" s="8" t="n"/>
+      <c r="I28" s="6" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2441,9 +2462,10 @@
           <t>16C00120</t>
         </is>
       </c>
-      <c r="B29" s="2">
-        <f>VLOOKUP(A29,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>FRD B/T</t>
+        </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
@@ -2465,13 +2487,13 @@
           <t>front grill broken</t>
         </is>
       </c>
-      <c r="G29" s="8" t="n">
+      <c r="G29" s="6" t="n">
         <v>45315</v>
       </c>
       <c r="H29" s="3" t="n">
         <v>572.51</v>
       </c>
-      <c r="I29" s="8" t="n">
+      <c r="I29" s="6" t="n">
         <v>45330</v>
       </c>
     </row>
@@ -2481,9 +2503,10 @@
           <t>16B00105</t>
         </is>
       </c>
-      <c r="B30" s="2">
-        <f>VLOOKUP(A30,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>FRD/VAN</t>
+        </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
@@ -2505,13 +2528,13 @@
           <t>unreported damage to left door, interior panel damaged, rear sliding door damaged, don’t bill for passenger door panel</t>
         </is>
       </c>
-      <c r="G30" s="8" t="n">
+      <c r="G30" s="6" t="n">
         <v>45359</v>
       </c>
       <c r="H30" s="3" t="n">
         <v>2290.59</v>
       </c>
-      <c r="I30" s="8" t="n">
+      <c r="I30" s="6" t="n">
         <v>45398</v>
       </c>
     </row>
@@ -2521,9 +2544,10 @@
           <t>16B00100</t>
         </is>
       </c>
-      <c r="B31" s="2">
-        <f>VLOOKUP(A31,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>FRD/VAN</t>
+        </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
@@ -2545,13 +2569,13 @@
           <t>SLIDING DOOR DENTED AND WONT CLOSE PROPERLY, UNREPORTED DAMAGE</t>
         </is>
       </c>
-      <c r="G31" s="8" t="n">
+      <c r="G31" s="6" t="n">
         <v>45359</v>
       </c>
       <c r="H31" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="I31" s="8" t="n"/>
+      <c r="I31" s="6" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2559,9 +2583,10 @@
           <t>16B00105</t>
         </is>
       </c>
-      <c r="B32" s="2">
-        <f>VLOOKUP(A32,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>FRD/VAN</t>
+        </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
@@ -2583,13 +2608,13 @@
           <t>taillight broken`</t>
         </is>
       </c>
-      <c r="G32" s="8" t="n">
+      <c r="G32" s="6" t="n">
         <v>45359</v>
       </c>
       <c r="H32" s="3" t="n">
         <v>391.32</v>
       </c>
-      <c r="I32" s="8" t="n">
+      <c r="I32" s="6" t="n">
         <v>45390</v>
       </c>
     </row>
@@ -2599,9 +2624,10 @@
           <t>16C00120</t>
         </is>
       </c>
-      <c r="B33" s="2">
-        <f>VLOOKUP(A33,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>FRD B/T</t>
+        </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
@@ -2623,13 +2649,13 @@
           <t>FRONT TIRES HAVE EXTREME WEAR</t>
         </is>
       </c>
-      <c r="G33" s="8" t="n">
+      <c r="G33" s="6" t="n">
         <v>45394</v>
       </c>
       <c r="H33" s="3" t="n">
         <v>450.68</v>
       </c>
-      <c r="I33" s="8" t="n">
+      <c r="I33" s="6" t="n">
         <v>45455</v>
       </c>
     </row>
@@ -2639,9 +2665,10 @@
           <t>16B00106</t>
         </is>
       </c>
-      <c r="B34" s="2">
-        <f>VLOOKUP(A34,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>FRD/VAN</t>
+        </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
@@ -2663,13 +2690,13 @@
           <t>WIND DAMAGE TO BACK P/S DOOR</t>
         </is>
       </c>
-      <c r="G34" s="8" t="n">
+      <c r="G34" s="6" t="n">
         <v>45398</v>
       </c>
       <c r="H34" s="3" t="n">
         <v>706.85</v>
       </c>
-      <c r="I34" s="8" t="n">
+      <c r="I34" s="6" t="n">
         <v>45440</v>
       </c>
     </row>
@@ -2679,9 +2706,10 @@
           <t>16B00102</t>
         </is>
       </c>
-      <c r="B35" s="2">
-        <f>VLOOKUP(A35,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>FRD/VAN</t>
+        </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
@@ -2703,13 +2731,13 @@
           <t>P/S MIRROR AND CORNER PANEL DAMAGED</t>
         </is>
       </c>
-      <c r="G35" s="8" t="n">
+      <c r="G35" s="6" t="n">
         <v>45413</v>
       </c>
       <c r="H35" s="3" t="n">
         <v>1182.72</v>
       </c>
-      <c r="I35" s="8" t="n">
+      <c r="I35" s="6" t="n">
         <v>45443</v>
       </c>
     </row>
@@ -2719,9 +2747,10 @@
           <t>16B00099</t>
         </is>
       </c>
-      <c r="B36" s="2">
-        <f>VLOOKUP(A36,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>FRD/VAN</t>
+        </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
@@ -2743,13 +2772,13 @@
           <t>LT REAR TOP CORNER, LT REAR CORNER PANEL SCRAP.</t>
         </is>
       </c>
-      <c r="G36" s="8" t="n">
+      <c r="G36" s="6" t="n">
         <v>45420</v>
       </c>
       <c r="H36" s="3" t="n">
         <v>6392.38</v>
       </c>
-      <c r="I36" s="8" t="n"/>
+      <c r="I36" s="6" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2757,9 +2786,10 @@
           <t>15B00066</t>
         </is>
       </c>
-      <c r="B37" s="2">
-        <f>VLOOKUP(A37,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>DOD P/U</t>
+        </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
@@ -2781,13 +2811,13 @@
           <t>WIND DAMAGE TO P/S DOOR</t>
         </is>
       </c>
-      <c r="G37" s="8" t="n">
+      <c r="G37" s="6" t="n">
         <v>45447</v>
       </c>
       <c r="H37" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I37" s="8" t="n"/>
+      <c r="I37" s="6" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2795,9 +2825,10 @@
           <t>16C00110</t>
         </is>
       </c>
-      <c r="B38" s="2">
-        <f>VLOOKUP(A38,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>FRD B/T</t>
+        </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
@@ -2819,13 +2850,13 @@
           <t>DOOR CHECKS DAMAGE, D/S DOOR HINGE AND PANEL BENT, P/S REAR FENDER BENT</t>
         </is>
       </c>
-      <c r="G38" s="8" t="n">
+      <c r="G38" s="6" t="n">
         <v>45498</v>
       </c>
       <c r="H38" s="3" t="n">
         <v>470.45</v>
       </c>
-      <c r="I38" s="8" t="n">
+      <c r="I38" s="6" t="n">
         <v>45552</v>
       </c>
     </row>
@@ -2835,9 +2866,10 @@
           <t>16C00104</t>
         </is>
       </c>
-      <c r="B39" s="2">
-        <f>VLOOKUP(A39,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>FRD B/T</t>
+        </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
@@ -2859,13 +2891,13 @@
           <t>D/S DOOR CHECKS, HINGES, AND PANEL DAMAGED</t>
         </is>
       </c>
-      <c r="G39" s="8" t="n">
+      <c r="G39" s="6" t="n">
         <v>45503</v>
       </c>
       <c r="H39" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I39" s="8" t="n"/>
+      <c r="I39" s="6" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2873,9 +2905,10 @@
           <t>16C00107</t>
         </is>
       </c>
-      <c r="B40" s="2">
-        <f>VLOOKUP(A40,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>FRD B/T</t>
+        </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
@@ -2897,13 +2930,13 @@
           <t>DAMAGE TO DOOR CHECKS ON BOTH DOORS (WIND DAMAGE) AND DIMPLES ON DOOR (WAIVER)</t>
         </is>
       </c>
-      <c r="G40" s="8" t="n">
+      <c r="G40" s="6" t="n">
         <v>45505</v>
       </c>
       <c r="H40" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I40" s="8" t="n"/>
+      <c r="I40" s="6" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2911,9 +2944,10 @@
           <t>16B00114</t>
         </is>
       </c>
-      <c r="B41" s="2">
-        <f>VLOOKUP(A41,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>FRD/VAN</t>
+        </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
@@ -2935,13 +2969,13 @@
           <t>ROOF DAMAGED BY OVERHANG</t>
         </is>
       </c>
-      <c r="G41" s="8" t="n">
+      <c r="G41" s="6" t="n">
         <v>45539</v>
       </c>
       <c r="H41" s="3" t="n">
         <v>67.5</v>
       </c>
-      <c r="I41" s="8" t="n">
+      <c r="I41" s="6" t="n">
         <v>45552</v>
       </c>
     </row>
@@ -2951,9 +2985,10 @@
           <t>16B00115</t>
         </is>
       </c>
-      <c r="B42" s="2">
-        <f>VLOOKUP(A42,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>FRD/VAN</t>
+        </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
@@ -2975,13 +3010,13 @@
           <t>RAN OVER SPIKE STRIP AT ECP (TIRE ONLY)</t>
         </is>
       </c>
-      <c r="G42" s="8" t="n">
+      <c r="G42" s="6" t="n">
         <v>45540</v>
       </c>
       <c r="H42" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I42" s="8" t="n"/>
+      <c r="I42" s="6" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2989,9 +3024,10 @@
           <t>18E00034</t>
         </is>
       </c>
-      <c r="B43" s="2">
-        <f>VLOOKUP(A43,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>F/L 20K</t>
+        </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
@@ -3013,13 +3049,13 @@
           <t xml:space="preserve">MINOR DAMAGE TO HEADLIGHT BRAcKET, WELDED TOGETHER IN 5 MINUTES </t>
         </is>
       </c>
-      <c r="G43" s="8" t="n">
+      <c r="G43" s="6" t="n">
         <v>45386</v>
       </c>
       <c r="H43" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I43" s="8" t="n"/>
+      <c r="I43" s="6" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3027,9 +3063,10 @@
           <t>05E00241</t>
         </is>
       </c>
-      <c r="B44" s="2">
-        <f>VLOOKUP(A44,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>HYS FL6</t>
+        </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
@@ -3051,13 +3088,13 @@
           <t>D/S WINDOW SHATTERED, D/S WINDOW TRACK</t>
         </is>
       </c>
-      <c r="G44" s="8" t="n">
+      <c r="G44" s="6" t="n">
         <v>45391</v>
       </c>
       <c r="H44" s="3" t="n">
         <v>150</v>
       </c>
-      <c r="I44" s="8" t="n"/>
+      <c r="I44" s="6" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3065,9 +3102,10 @@
           <t>10B02055</t>
         </is>
       </c>
-      <c r="B45" s="2">
-        <f>VLOOKUP(A45,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>CHE MLT</t>
+        </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
@@ -3089,13 +3127,13 @@
           <t>D/S WING DAMAGE</t>
         </is>
       </c>
-      <c r="G45" s="8" t="n">
+      <c r="G45" s="6" t="n">
         <v>45566</v>
       </c>
       <c r="H45" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I45" s="8" t="n"/>
+      <c r="I45" s="6" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3103,9 +3141,10 @@
           <t>10B02056</t>
         </is>
       </c>
-      <c r="B46" s="2">
-        <f>VLOOKUP(A46,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>CHE MLT</t>
+        </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
@@ -3127,13 +3166,13 @@
           <t>BREAK BOOSTER, NO POWER STEERING, NO COOLANT</t>
         </is>
       </c>
-      <c r="G46" s="8" t="n">
+      <c r="G46" s="6" t="n">
         <v>45566</v>
       </c>
       <c r="H46" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I46" s="8" t="n"/>
+      <c r="I46" s="6" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3141,9 +3180,10 @@
           <t>11B01322</t>
         </is>
       </c>
-      <c r="B47" s="2">
-        <f>VLOOKUP(A47,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>CHE MLT</t>
+        </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
@@ -3165,13 +3205,13 @@
           <t>D/S WINDOW DOOR CRANK BROKEN OFF</t>
         </is>
       </c>
-      <c r="G47" s="8" t="n">
+      <c r="G47" s="6" t="n">
         <v>45566</v>
       </c>
       <c r="H47" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I47" s="8" t="n"/>
+      <c r="I47" s="6" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3179,9 +3219,10 @@
           <t>11B01403</t>
         </is>
       </c>
-      <c r="B48" s="2">
-        <f>VLOOKUP(A48,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>CHE MLT</t>
+        </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
@@ -3203,13 +3244,13 @@
           <t xml:space="preserve">WIND DAMAGE  </t>
         </is>
       </c>
-      <c r="G48" s="8" t="n">
+      <c r="G48" s="6" t="n">
         <v>45566</v>
       </c>
       <c r="H48" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I48" s="8" t="n"/>
+      <c r="I48" s="6" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3217,9 +3258,10 @@
           <t>11B01317</t>
         </is>
       </c>
-      <c r="B49" s="2">
-        <f>VLOOKUP(A49,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>CHE MLT</t>
+        </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
@@ -3241,13 +3283,13 @@
           <t>WIND DAMAGE P/S DOOR, LEFT REAR DOOR LOWER HINGE</t>
         </is>
       </c>
-      <c r="G49" s="8" t="n">
+      <c r="G49" s="6" t="n">
         <v>45566</v>
       </c>
       <c r="H49" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I49" s="8" t="n"/>
+      <c r="I49" s="6" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3255,9 +3297,10 @@
           <t>10B01703</t>
         </is>
       </c>
-      <c r="B50" s="2">
-        <f>VLOOKUP(A50,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>CHE P/U</t>
+        </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
@@ -3279,13 +3322,13 @@
           <t>P/S REAR BOX AND TAIL LIGHT</t>
         </is>
       </c>
-      <c r="G50" s="8" t="n">
+      <c r="G50" s="6" t="n">
         <v>45566</v>
       </c>
       <c r="H50" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I50" s="8" t="n"/>
+      <c r="I50" s="6" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3293,9 +3336,10 @@
           <t>10B02062</t>
         </is>
       </c>
-      <c r="B51" s="2">
-        <f>VLOOKUP(A51,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>CHE MLT</t>
+        </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
@@ -3317,13 +3361,13 @@
           <t>PENCIL HOLES IN DASH, ASSIST HANDLE BY SLIDING DOOR, P/S AND D/S WIND DAMAGE</t>
         </is>
       </c>
-      <c r="G51" s="8" t="n">
+      <c r="G51" s="6" t="n">
         <v>45566</v>
       </c>
       <c r="H51" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I51" s="8" t="n"/>
+      <c r="I51" s="6" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3331,9 +3375,10 @@
           <t>16B00102</t>
         </is>
       </c>
-      <c r="B52" s="2">
-        <f>VLOOKUP(A52,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>FRD/VAN</t>
+        </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
@@ -3355,13 +3400,13 @@
           <t>WIND DAMAGE TO D/S &amp; P/S DOORS</t>
         </is>
       </c>
-      <c r="G52" s="8" t="n">
+      <c r="G52" s="6" t="n">
         <v>45573</v>
       </c>
       <c r="H52" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I52" s="8" t="n"/>
+      <c r="I52" s="6" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3369,9 +3414,10 @@
           <t>16B00106</t>
         </is>
       </c>
-      <c r="B53" s="2">
-        <f>VLOOKUP(A53,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>FRD/VAN</t>
+        </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
@@ -3393,13 +3439,13 @@
           <t>DAMAGE TO D/S DOOR, PANEL, HARNESS, MIRROR, DOOR CHECK AND P/S DOOR AND MIRROR HOUSING</t>
         </is>
       </c>
-      <c r="G53" s="8" t="n">
+      <c r="G53" s="6" t="n">
         <v>45575</v>
       </c>
       <c r="H53" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I53" s="8" t="n"/>
+      <c r="I53" s="6" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3407,9 +3453,10 @@
           <t>10B02067</t>
         </is>
       </c>
-      <c r="B54" s="2">
-        <f>VLOOKUP(A54,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>CHE MLT</t>
+        </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
@@ -3431,13 +3478,13 @@
           <t>BROKE SLIDING DOOR GLASS</t>
         </is>
       </c>
-      <c r="G54" s="8" t="n">
+      <c r="G54" s="6" t="n">
         <v>45580</v>
       </c>
       <c r="H54" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I54" s="8" t="n"/>
+      <c r="I54" s="6" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3445,9 +3492,10 @@
           <t>07B00702</t>
         </is>
       </c>
-      <c r="B55" s="2">
-        <f>VLOOKUP(A55,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>FRD P/U</t>
+        </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
@@ -3469,13 +3517,13 @@
           <t>PLUGGED DPF</t>
         </is>
       </c>
-      <c r="G55" s="8" t="n">
+      <c r="G55" s="6" t="n">
         <v>45595</v>
       </c>
       <c r="H55" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I55" s="8" t="n"/>
+      <c r="I55" s="6" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -3508,13 +3556,13 @@
           <t>SHATTERED WINDSHIELD, WIPER ARM</t>
         </is>
       </c>
-      <c r="G56" s="8" t="n">
+      <c r="G56" s="6" t="n">
         <v>45629</v>
       </c>
       <c r="H56" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I56" s="8" t="n"/>
+      <c r="I56" s="6" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -3522,9 +3570,10 @@
           <t>07B00135</t>
         </is>
       </c>
-      <c r="B57" s="2">
-        <f>VLOOKUP(A57,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>FTL TRC</t>
+        </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
@@ -3546,11 +3595,11 @@
           <t>FIFTH WHEEL PLATE WORN DOWN, NOT GREASED</t>
         </is>
       </c>
-      <c r="G57" s="8" t="n">
+      <c r="G57" s="6" t="n">
         <v>45635</v>
       </c>
       <c r="H57" s="3" t="n"/>
-      <c r="I57" s="8" t="n"/>
+      <c r="I57" s="6" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -3558,9 +3607,10 @@
           <t>16B00362</t>
         </is>
       </c>
-      <c r="B58" s="2">
-        <f>VLOOKUP(A58,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>CHE PU</t>
+        </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
@@ -3582,13 +3632,13 @@
           <t>REAR BUMBER DENT LEFT SIDE</t>
         </is>
       </c>
-      <c r="G58" s="8" t="n">
+      <c r="G58" s="6" t="n">
         <v>45643</v>
       </c>
       <c r="H58" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I58" s="8" t="n"/>
+      <c r="I58" s="6" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -3596,9 +3646,10 @@
           <t>16B00109</t>
         </is>
       </c>
-      <c r="B59" s="2">
-        <f>VLOOKUP(A59,'[1]PCN23 Query'!$1:$1048576,5,FALSE)</f>
-        <v/>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>FRD/VAN</t>
+        </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
@@ -3620,13 +3671,13 @@
           <t>DENT REAR PASSENGER SIDE NEAR WHEEL WELL</t>
         </is>
       </c>
-      <c r="G59" s="8" t="n">
+      <c r="G59" s="6" t="n">
         <v>45649</v>
       </c>
       <c r="H59" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I59" s="8" t="n"/>
+      <c r="I59" s="6" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -3659,13 +3710,13 @@
           <t>EXHAUST STACK</t>
         </is>
       </c>
-      <c r="G60" s="8" t="n">
+      <c r="G60" s="6" t="n">
         <v>45358</v>
       </c>
       <c r="H60" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I60" s="8" t="n"/>
+      <c r="I60" s="6" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -3698,13 +3749,13 @@
           <t>D/S WINDOW SHATTERED, D/S WINDOW TRACK</t>
         </is>
       </c>
-      <c r="G61" s="8" t="n">
+      <c r="G61" s="6" t="n">
         <v>45391</v>
       </c>
       <c r="H61" s="3" t="n">
         <v>150</v>
       </c>
-      <c r="I61" s="8" t="n"/>
+      <c r="I61" s="6" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -3737,13 +3788,13 @@
           <t>D/S BACK STEP BENT</t>
         </is>
       </c>
-      <c r="G62" s="8" t="n">
+      <c r="G62" s="6" t="n">
         <v>45531</v>
       </c>
       <c r="H62" s="3" t="n">
         <v>1164</v>
       </c>
-      <c r="I62" s="8" t="n">
+      <c r="I62" s="6" t="n">
         <v>45601</v>
       </c>
     </row>
@@ -3778,13 +3829,13 @@
           <t>BREAK BOOSTER, NO POWER STEERING, NO COOLANT</t>
         </is>
       </c>
-      <c r="G63" s="8" t="n">
+      <c r="G63" s="6" t="n">
         <v>45566</v>
       </c>
       <c r="H63" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I63" s="8" t="n"/>
+      <c r="I63" s="6" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -3817,13 +3868,13 @@
           <t>D/S WINDOW DOOR CRANK BROKEN OFF</t>
         </is>
       </c>
-      <c r="G64" s="8" t="n">
+      <c r="G64" s="6" t="n">
         <v>45566</v>
       </c>
       <c r="H64" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I64" s="8" t="n"/>
+      <c r="I64" s="6" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -3856,13 +3907,13 @@
           <t>P/S REAR BOX AND TAIL LIGHT</t>
         </is>
       </c>
-      <c r="G65" s="8" t="n">
+      <c r="G65" s="6" t="n">
         <v>45566</v>
       </c>
       <c r="H65" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I65" s="8" t="n"/>
+      <c r="I65" s="6" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -3895,13 +3946,13 @@
           <t>WIND DAMAGE TO D/S &amp; P/S DOORS</t>
         </is>
       </c>
-      <c r="G66" s="8" t="n">
+      <c r="G66" s="6" t="n">
         <v>45573</v>
       </c>
       <c r="H66" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I66" s="8" t="n"/>
+      <c r="I66" s="6" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -3934,13 +3985,13 @@
           <t>DAMAGE TO D/S DOOR, PANEL, HARNESS, MIRROR, DOOR CHECK AND P/S DOOR AND MIRROR HOUSING</t>
         </is>
       </c>
-      <c r="G67" s="8" t="n">
+      <c r="G67" s="6" t="n">
         <v>45575</v>
       </c>
       <c r="H67" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I67" s="8" t="n"/>
+      <c r="I67" s="6" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -3973,13 +4024,13 @@
           <t>PLUGGED DPF</t>
         </is>
       </c>
-      <c r="G68" s="8" t="n">
+      <c r="G68" s="6" t="n">
         <v>45595</v>
       </c>
       <c r="H68" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I68" s="8" t="n"/>
+      <c r="I68" s="6" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -4012,13 +4063,13 @@
           <t>SHATTERED WINDSHIELD, WIPER ARM</t>
         </is>
       </c>
-      <c r="G69" s="8" t="n">
+      <c r="G69" s="6" t="n">
         <v>45629</v>
       </c>
       <c r="H69" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I69" s="8" t="n"/>
+      <c r="I69" s="6" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -4051,13 +4102,13 @@
           <t xml:space="preserve">Passenger's rear quarter panel damaged and rear door </t>
         </is>
       </c>
-      <c r="G70" s="8" t="n">
+      <c r="G70" s="6" t="n">
         <v>45629</v>
       </c>
       <c r="H70" s="3" t="n">
         <v>2158.49</v>
       </c>
-      <c r="I70" s="8" t="n"/>
+      <c r="I70" s="6" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -4090,11 +4141,11 @@
           <t>FIFTH WHEEL PLATE WORN DOWN, NOT GREASED</t>
         </is>
       </c>
-      <c r="G71" s="8" t="n">
+      <c r="G71" s="6" t="n">
         <v>45635</v>
       </c>
       <c r="H71" s="3" t="n"/>
-      <c r="I71" s="8" t="n"/>
+      <c r="I71" s="6" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -4127,13 +4178,13 @@
           <t>REAR BUMBER DENT LEFT SIDE</t>
         </is>
       </c>
-      <c r="G72" s="8" t="n">
+      <c r="G72" s="6" t="n">
         <v>45643</v>
       </c>
       <c r="H72" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I72" s="8" t="n"/>
+      <c r="I72" s="6" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -4166,13 +4217,13 @@
           <t>DENT REAR PASSENGER SIDE NEAR WHEEL WELL</t>
         </is>
       </c>
-      <c r="G73" s="8" t="n">
+      <c r="G73" s="6" t="n">
         <v>45649</v>
       </c>
       <c r="H73" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I73" s="8" t="n"/>
+      <c r="I73" s="6" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -4205,13 +4256,13 @@
           <t>RT REAR FENDER GOUGE, DAMAGE PAINT, RT REAR REFLECTOR DAMAGED</t>
         </is>
       </c>
-      <c r="G74" s="8" t="n">
+      <c r="G74" s="6" t="n">
         <v>45680</v>
       </c>
       <c r="H74" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I74" s="8" t="n"/>
+      <c r="I74" s="6" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -4244,13 +4295,13 @@
           <t>Broken Driver's side view mirror</t>
         </is>
       </c>
-      <c r="G75" s="8" t="n">
+      <c r="G75" s="6" t="n">
         <v>45685</v>
       </c>
       <c r="H75" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I75" s="8" t="n"/>
+      <c r="I75" s="6" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -4283,13 +4334,13 @@
           <t>Front grill, front bumper, front pintle hook, rf front fender</t>
         </is>
       </c>
-      <c r="G76" s="8" t="n">
+      <c r="G76" s="6" t="n">
         <v>45686</v>
       </c>
       <c r="H76" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I76" s="8" t="n"/>
+      <c r="I76" s="6" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -4322,13 +4373,13 @@
           <t xml:space="preserve">REAR BUMPER, RH REAR SIDE PANEL </t>
         </is>
       </c>
-      <c r="G77" s="8" t="n">
+      <c r="G77" s="6" t="n">
         <v>45686</v>
       </c>
       <c r="H77" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I77" s="8" t="n"/>
+      <c r="I77" s="6" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -4361,13 +4412,13 @@
           <t>D/S DOOR HANDLE BROKEN-17 Sept not reported</t>
         </is>
       </c>
-      <c r="G78" s="8" t="n">
+      <c r="G78" s="6" t="n">
         <v>45688</v>
       </c>
       <c r="H78" s="3" t="n">
         <v>810</v>
       </c>
-      <c r="I78" s="8" t="n"/>
+      <c r="I78" s="6" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -4400,13 +4451,13 @@
           <t>FRONT WINDSHIELD BROKEN</t>
         </is>
       </c>
-      <c r="G79" s="8" t="n">
+      <c r="G79" s="6" t="n">
         <v>45699</v>
       </c>
       <c r="H79" s="3" t="n">
         <v>91.70999999999999</v>
       </c>
-      <c r="I79" s="8" t="n"/>
+      <c r="I79" s="6" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -4439,13 +4490,13 @@
           <t xml:space="preserve">Interior Damage, (Seat and Dash) </t>
         </is>
       </c>
-      <c r="G80" s="8" t="n">
+      <c r="G80" s="6" t="n">
         <v>45700</v>
       </c>
       <c r="H80" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I80" s="8" t="n"/>
+      <c r="I80" s="6" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -4478,13 +4529,13 @@
           <t xml:space="preserve">WIND DAMAGE D/S DOOR, D/S FENDER, GAS DOOR </t>
         </is>
       </c>
-      <c r="G81" s="8" t="n">
+      <c r="G81" s="6" t="n">
         <v>45699</v>
       </c>
       <c r="H81" s="3" t="n">
         <v>3910.52</v>
       </c>
-      <c r="I81" s="8" t="n"/>
+      <c r="I81" s="6" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -4517,13 +4568,13 @@
           <t>REIGHT REAR TAIL LIGHT BROKEN AND DAMAGE AROUND THE LIGHT (METAL WORK)</t>
         </is>
       </c>
-      <c r="G82" s="8" t="n">
+      <c r="G82" s="6" t="n">
         <v>45715</v>
       </c>
       <c r="H82" s="3" t="n">
         <v>2055.6</v>
       </c>
-      <c r="I82" s="8" t="n"/>
+      <c r="I82" s="6" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -4556,13 +4607,13 @@
           <t>DAMAGE TO BUMPER AND SIDE FENDER</t>
         </is>
       </c>
-      <c r="G83" s="8" t="n">
+      <c r="G83" s="6" t="n">
         <v>45715</v>
       </c>
       <c r="H83" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I83" s="8" t="n"/>
+      <c r="I83" s="6" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -4595,13 +4646,13 @@
           <t>P/S MIRROR</t>
         </is>
       </c>
-      <c r="G84" s="8" t="n">
+      <c r="G84" s="6" t="n">
         <v>45723</v>
       </c>
       <c r="H84" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I84" s="8" t="n"/>
+      <c r="I84" s="6" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -4634,13 +4685,13 @@
           <t>P/S MIRROR</t>
         </is>
       </c>
-      <c r="G85" s="8" t="n">
+      <c r="G85" s="6" t="n">
         <v>45726</v>
       </c>
       <c r="H85" s="3" t="n">
         <v>30.87</v>
       </c>
-      <c r="I85" s="8" t="n"/>
+      <c r="I85" s="6" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -4673,13 +4724,13 @@
           <t>REAR WINDOW BROKEN</t>
         </is>
       </c>
-      <c r="G86" s="8" t="n">
+      <c r="G86" s="6" t="n">
         <v>45768</v>
       </c>
       <c r="H86" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I86" s="8" t="n"/>
+      <c r="I86" s="6" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -4712,13 +4763,13 @@
           <t>WIND DAMAGE PASSENGER DOOR, A-Pillar Damage</t>
         </is>
       </c>
-      <c r="G87" s="8" t="n">
+      <c r="G87" s="6" t="n">
         <v>45782</v>
       </c>
       <c r="H87" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I87" s="8" t="n"/>
+      <c r="I87" s="6" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -4751,13 +4802,13 @@
           <t>BROKEN LEFT DOOR WINDOW</t>
         </is>
       </c>
-      <c r="G88" s="8" t="n">
+      <c r="G88" s="6" t="n">
         <v>45789</v>
       </c>
       <c r="H88" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I88" s="8" t="n"/>
+      <c r="I88" s="6" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -4790,13 +4841,13 @@
           <t xml:space="preserve">WIND DAMAGE BOTH DOORS, BOTH FRONT FENDERS, BOX SIDE WINDOW BROKEN, SLIDING DOOR BROKEN, </t>
         </is>
       </c>
-      <c r="G89" s="8" t="n">
+      <c r="G89" s="6" t="n">
         <v>45792</v>
       </c>
       <c r="H89" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I89" s="8" t="n"/>
+      <c r="I89" s="6" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -4829,13 +4880,13 @@
           <t>WIND DAMAGE TO PASSENGER DOOR AND FENDER</t>
         </is>
       </c>
-      <c r="G90" s="8" t="n">
+      <c r="G90" s="6" t="n">
         <v>45796</v>
       </c>
       <c r="H90" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I90" s="8" t="n"/>
+      <c r="I90" s="6" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -4868,13 +4919,13 @@
           <t>PASS SIDE HOOD/FENDER DAMAGED</t>
         </is>
       </c>
-      <c r="G91" s="8" t="n">
+      <c r="G91" s="6" t="n">
         <v>45806</v>
       </c>
       <c r="H91" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I91" s="8" t="n"/>
+      <c r="I91" s="6" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -4907,13 +4958,13 @@
           <t>WIND DAMAGE BOTH DOORS, SLIDING DOOR, WIRE HARNESS COVER, STEP ACCESS PLATE</t>
         </is>
       </c>
-      <c r="G92" s="8" t="n">
+      <c r="G92" s="6" t="n">
         <v>45817</v>
       </c>
       <c r="H92" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I92" s="8" t="n"/>
+      <c r="I92" s="6" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -4946,13 +4997,13 @@
           <t>LEFT REAR QUATER PANEL</t>
         </is>
       </c>
-      <c r="G93" s="8" t="n">
+      <c r="G93" s="6" t="n">
         <v>45817</v>
       </c>
       <c r="H93" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I93" s="8" t="n"/>
+      <c r="I93" s="6" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -4985,13 +5036,13 @@
           <t>RIGHT FRONT FENDER, GRILL AND HOOD</t>
         </is>
       </c>
-      <c r="G94" s="8" t="n">
+      <c r="G94" s="6" t="n">
         <v>45824</v>
       </c>
       <c r="H94" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I94" s="8" t="n"/>
+      <c r="I94" s="6" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -5024,11 +5075,11 @@
           <t>WIND DAMAGE BOTH DOORS, A PILLARS</t>
         </is>
       </c>
-      <c r="G95" s="8" t="n">
+      <c r="G95" s="6" t="n">
         <v>45832</v>
       </c>
       <c r="H95" s="3" t="n"/>
-      <c r="I95" s="8" t="n"/>
+      <c r="I95" s="6" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -5059,13 +5110,13 @@
           <t>TIRE</t>
         </is>
       </c>
-      <c r="G96" s="8" t="n">
+      <c r="G96" s="6" t="n">
         <v>45833</v>
       </c>
       <c r="H96" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I96" s="8" t="n"/>
+      <c r="I96" s="6" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -5098,13 +5149,13 @@
           <t>Rear Bumper</t>
         </is>
       </c>
-      <c r="G97" s="8" t="n">
+      <c r="G97" s="6" t="n">
         <v>45838</v>
       </c>
       <c r="H97" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I97" s="8" t="n"/>
+      <c r="I97" s="6" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -5135,13 +5186,13 @@
           <t xml:space="preserve">FLAT TIRES </t>
         </is>
       </c>
-      <c r="G98" s="8" t="n">
+      <c r="G98" s="6" t="n">
         <v>45839</v>
       </c>
       <c r="H98" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I98" s="8" t="n"/>
+      <c r="I98" s="6" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -5174,13 +5225,13 @@
           <t>BENT FRAME/RAILS</t>
         </is>
       </c>
-      <c r="G99" s="8" t="n">
+      <c r="G99" s="6" t="n">
         <v>45839</v>
       </c>
       <c r="H99" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I99" s="8" t="n"/>
+      <c r="I99" s="6" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -5211,11 +5262,11 @@
           <t>PAINT AND METAL SCUFFS</t>
         </is>
       </c>
-      <c r="G100" s="8" t="n">
+      <c r="G100" s="6" t="n">
         <v>45861</v>
       </c>
       <c r="H100" s="3" t="n"/>
-      <c r="I100" s="8" t="n"/>
+      <c r="I100" s="6" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -5248,13 +5299,13 @@
           <t>DENTS FRONT BUMPER</t>
         </is>
       </c>
-      <c r="G101" s="8" t="n">
+      <c r="G101" s="6" t="n">
         <v>45861</v>
       </c>
       <c r="H101" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I101" s="8" t="n"/>
+      <c r="I101" s="6" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -5287,11 +5338,11 @@
           <t>WIND DAMAGE BOTH DOORS, A PILLARS AND BOTH FRONT FENDERS</t>
         </is>
       </c>
-      <c r="G102" s="8" t="n">
+      <c r="G102" s="6" t="n">
         <v>45861</v>
       </c>
       <c r="H102" s="3" t="n"/>
-      <c r="I102" s="8" t="n"/>
+      <c r="I102" s="6" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -5324,13 +5375,13 @@
           <t>DENT AND BROKEN REAR DOOR HANDLE</t>
         </is>
       </c>
-      <c r="G103" s="8" t="n">
+      <c r="G103" s="6" t="n">
         <v>45862</v>
       </c>
       <c r="H103" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I103" s="8" t="n"/>
+      <c r="I103" s="6" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -5363,13 +5414,13 @@
           <t>DENT IN CAB</t>
         </is>
       </c>
-      <c r="G104" s="8" t="n">
+      <c r="G104" s="6" t="n">
         <v>45868</v>
       </c>
       <c r="H104" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I104" s="8" t="n"/>
+      <c r="I104" s="6" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -5402,13 +5453,13 @@
           <t xml:space="preserve">AIR VENTS, CENTER CONSOLE, REAR TAIL LIGHT </t>
         </is>
       </c>
-      <c r="G105" s="8" t="n">
+      <c r="G105" s="6" t="n">
         <v>45868</v>
       </c>
       <c r="H105" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I105" s="8" t="n"/>
+      <c r="I105" s="6" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -5441,11 +5492,11 @@
           <t>WIND DAMAGE BOTH DOORS, A PILLARS</t>
         </is>
       </c>
-      <c r="G106" s="8" t="n">
+      <c r="G106" s="6" t="n">
         <v>45873</v>
       </c>
       <c r="H106" s="3" t="n"/>
-      <c r="I106" s="8" t="n"/>
+      <c r="I106" s="6" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -5476,13 +5527,13 @@
           <t>WATER HEATER AND WINTERIZATION SINGLE PHASE OUTLETS ARE BROKEN</t>
         </is>
       </c>
-      <c r="G107" s="8" t="n">
+      <c r="G107" s="6" t="n">
         <v>45889</v>
       </c>
       <c r="H107" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I107" s="8" t="n"/>
+      <c r="I107" s="6" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -5515,13 +5566,13 @@
           <t>FUEL DOOR</t>
         </is>
       </c>
-      <c r="G108" s="8" t="n">
+      <c r="G108" s="6" t="n">
         <v>45894</v>
       </c>
       <c r="H108" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I108" s="8" t="n"/>
+      <c r="I108" s="6" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -5554,13 +5605,13 @@
           <t>DRIVER'S DOOR DAMAGED FROM ACCIDENT, HOLE IN AIRBAG COVER, PASS DOOR RIPPED AND DOOR HANDLE BROKEN</t>
         </is>
       </c>
-      <c r="G109" s="8" t="n">
+      <c r="G109" s="6" t="n">
         <v>45924</v>
       </c>
       <c r="H109" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I109" s="8" t="n"/>
+      <c r="I109" s="6" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -5593,13 +5644,13 @@
           <t>WIND DAMAGE BOTH DOORS, A PILLARS</t>
         </is>
       </c>
-      <c r="G110" s="8" t="n">
+      <c r="G110" s="6" t="n">
         <v>45925</v>
       </c>
       <c r="H110" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I110" s="8" t="n"/>
+      <c r="I110" s="6" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -5632,13 +5683,13 @@
           <t>WIND DAMAGE BOTH DOORS, A PILLARS, HOOD DENTED AND REAR DOOR METAL STRIP</t>
         </is>
       </c>
-      <c r="G111" s="8" t="n">
+      <c r="G111" s="6" t="n">
         <v>45925</v>
       </c>
       <c r="H111" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I111" s="8" t="n"/>
+      <c r="I111" s="6" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -5671,13 +5722,13 @@
           <t>WIND DAMAGE BOTH DOORS, A PILLARS</t>
         </is>
       </c>
-      <c r="G112" s="8" t="n">
+      <c r="G112" s="6" t="n">
         <v>45931</v>
       </c>
       <c r="H112" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I112" s="8" t="n"/>
+      <c r="I112" s="6" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -5710,13 +5761,13 @@
           <t>DENTED RIGHT REAR QUARTER PANEL, BROKE RIGHT REAR TAILLIGHT TABS</t>
         </is>
       </c>
-      <c r="G113" s="8" t="n">
+      <c r="G113" s="6" t="n">
         <v>45946</v>
       </c>
       <c r="H113" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I113" s="8" t="n"/>
+      <c r="I113" s="6" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -5749,13 +5800,13 @@
           <t>VEHICLE WAS DRIVEN ON A FLAT TIRE</t>
         </is>
       </c>
-      <c r="G114" s="8" t="n">
+      <c r="G114" s="6" t="n">
         <v>45953</v>
       </c>
       <c r="H114" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I114" s="8" t="n"/>
+      <c r="I114" s="6" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -5788,11 +5839,11 @@
           <t>BENT RIM</t>
         </is>
       </c>
-      <c r="G115" s="8" t="n">
+      <c r="G115" s="6" t="n">
         <v>45954</v>
       </c>
       <c r="H115" s="3" t="n"/>
-      <c r="I115" s="8" t="n"/>
+      <c r="I115" s="6" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -5825,11 +5876,11 @@
           <t>PASSENGER DOOR AND FENDER DAMAGE</t>
         </is>
       </c>
-      <c r="G116" s="8" t="n">
+      <c r="G116" s="6" t="n">
         <v>45966</v>
       </c>
       <c r="H116" s="3" t="n"/>
-      <c r="I116" s="8" t="n"/>
+      <c r="I116" s="6" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -5862,13 +5913,13 @@
           <t>REAR BUMPER, QUARTER PANEL AND TAIL LIGHT</t>
         </is>
       </c>
-      <c r="G117" s="8" t="n">
+      <c r="G117" s="6" t="n">
         <v>45975</v>
       </c>
       <c r="H117" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I117" s="8" t="n"/>
+      <c r="I117" s="6" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -5901,11 +5952,11 @@
           <t>BOTH DOORS HAVE WIND DAMAGE AND BOTH A-PILLERS</t>
         </is>
       </c>
-      <c r="G118" s="8" t="n">
+      <c r="G118" s="6" t="n">
         <v>45994</v>
       </c>
       <c r="H118" s="3" t="n"/>
-      <c r="I118" s="8" t="n"/>
+      <c r="I118" s="6" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -5938,13 +5989,13 @@
           <t>HOOD DENT, A-PILLARS, REAR DOOR</t>
         </is>
       </c>
-      <c r="G119" s="8" t="n">
+      <c r="G119" s="6" t="n">
         <v>46030</v>
       </c>
       <c r="H119" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="I119" s="8" t="n"/>
+      <c r="I119" s="6" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -5977,11 +6028,11 @@
           <t>P/S DOOR WINDOW</t>
         </is>
       </c>
-      <c r="G120" s="8" t="n">
+      <c r="G120" s="6" t="n">
         <v>46043</v>
       </c>
       <c r="H120" s="3" t="n"/>
-      <c r="I120" s="8" t="n"/>
+      <c r="I120" s="6" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -6014,11 +6065,11 @@
           <t>P/S DOOR AND FENDER</t>
         </is>
       </c>
-      <c r="G121" s="8" t="n">
+      <c r="G121" s="6" t="n">
         <v>46045</v>
       </c>
       <c r="H121" s="3" t="n"/>
-      <c r="I121" s="8" t="n"/>
+      <c r="I121" s="6" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -6051,11 +6102,11 @@
           <t>WIND DAMAGE TO BOTH DOORS, PS FRONT FENDER</t>
         </is>
       </c>
-      <c r="G122" s="8" t="n">
+      <c r="G122" s="6" t="n">
         <v>46048</v>
       </c>
       <c r="H122" s="3" t="n"/>
-      <c r="I122" s="8" t="n"/>
+      <c r="I122" s="6" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -6088,11 +6139,11 @@
           <t>WIND DAMAGE</t>
         </is>
       </c>
-      <c r="G123" s="8" t="n">
+      <c r="G123" s="6" t="n">
         <v>46076</v>
       </c>
       <c r="H123" s="3" t="n"/>
-      <c r="I123" s="8" t="n"/>
+      <c r="I123" s="6" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -6125,11 +6176,11 @@
           <t>SCUFF ON DRIVERS SIDE REAR BUMPER</t>
         </is>
       </c>
-      <c r="G124" s="8" t="n">
+      <c r="G124" s="6" t="n">
         <v>46097</v>
       </c>
       <c r="H124" s="3" t="n"/>
-      <c r="I124" s="8" t="n"/>
+      <c r="I124" s="6" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I124"/>

</xml_diff>